<commit_message>
Update: Local function to work
</commit_message>
<xml_diff>
--- a/public/templates/Plantilla_Preventivo.xlsx
+++ b/public/templates/Plantilla_Preventivo.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29910"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29917"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BAC1CCA1-EFCF-4CFC-B6AB-BE97950DDC31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7971BA34-0A84-4A28-B921-EB0E7B45B4CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,12 +31,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="73">
   <si>
     <t xml:space="preserve">Orden/Reporte de Servicio </t>
-  </si>
-  <si>
-    <t>MHOS-SSM-EL-0001</t>
   </si>
   <si>
     <t>Fecha</t>
@@ -246,6 +243,9 @@
   </si>
   <si>
     <t>Sello de la Unidad</t>
+  </si>
+  <si>
+    <t>MHOS-SSM-EL-0001</t>
   </si>
   <si>
     <t>Rutina de anexo técnico</t>
@@ -1473,7 +1473,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="161">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1537,6 +1537,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1588,9 +1595,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1618,9 +1622,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1628,9 +1629,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1723,6 +1721,33 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1738,30 +1763,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1789,13 +1790,97 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1825,94 +1910,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2250,34 +2247,32 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L191"/>
+  <dimension ref="A1:L192"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="0" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="26.42578125" customWidth="1"/>
-    <col min="3" max="3" width="25.7109375" customWidth="1"/>
+    <col min="3" max="3" width="26.7109375" customWidth="1"/>
     <col min="4" max="4" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="10.28515625" customWidth="1"/>
     <col min="8" max="8" width="0.28515625" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="16.7109375" customWidth="1"/>
+    <col min="10" max="10" width="8.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="33" customHeight="1"/>
-    <row r="3" spans="1:12" ht="33" customHeight="1"/>
+    <row r="1" spans="1:12" ht="30" customHeight="1"/>
+    <row r="3" spans="1:12" ht="30" customHeight="1"/>
     <row r="5" spans="1:12">
       <c r="A5" s="1"/>
       <c r="B5" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C5" s="2"/>
-      <c r="D5" s="148" t="s">
-        <v>1</v>
-      </c>
-      <c r="E5" s="149"/>
-      <c r="F5" s="150"/>
+      <c r="D5" s="120"/>
+      <c r="E5" s="121"/>
+      <c r="F5" s="122"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -2288,12 +2283,12 @@
     <row r="6" spans="1:12">
       <c r="A6" s="1"/>
       <c r="B6" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="113"/>
-      <c r="E6" s="160"/>
-      <c r="F6" s="160"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -2303,11 +2298,6 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="1"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
@@ -2318,37 +2308,37 @@
     <row r="8" spans="1:12">
       <c r="A8" s="1"/>
       <c r="B8" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" s="114"/>
-      <c r="D8" s="151"/>
-      <c r="E8" s="151"/>
-      <c r="F8" s="151"/>
-      <c r="G8" s="151"/>
-      <c r="H8" s="151"/>
-      <c r="I8" s="151"/>
-      <c r="J8" s="151"/>
-      <c r="K8" s="151"/>
-      <c r="L8" s="152"/>
+        <v>2</v>
+      </c>
+      <c r="C8" s="115"/>
+      <c r="D8" s="123"/>
+      <c r="E8" s="123"/>
+      <c r="F8" s="123"/>
+      <c r="G8" s="123"/>
+      <c r="H8" s="123"/>
+      <c r="I8" s="123"/>
+      <c r="J8" s="123"/>
+      <c r="K8" s="123"/>
+      <c r="L8" s="124"/>
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="1"/>
       <c r="B9" s="4"/>
-      <c r="C9" s="115"/>
-      <c r="D9" s="115"/>
-      <c r="E9" s="115"/>
-      <c r="F9" s="115"/>
-      <c r="G9" s="115"/>
-      <c r="H9" s="115"/>
-      <c r="I9" s="115"/>
-      <c r="J9" s="115"/>
-      <c r="K9" s="115"/>
-      <c r="L9" s="116"/>
+      <c r="C9" s="116"/>
+      <c r="D9" s="116"/>
+      <c r="E9" s="116"/>
+      <c r="F9" s="116"/>
+      <c r="G9" s="116"/>
+      <c r="H9" s="116"/>
+      <c r="I9" s="116"/>
+      <c r="J9" s="116"/>
+      <c r="K9" s="116"/>
+      <c r="L9" s="117"/>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="1"/>
       <c r="B10" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C10" s="70"/>
       <c r="D10" s="70"/>
@@ -2364,25 +2354,25 @@
     <row r="11" spans="1:12">
       <c r="A11" s="1"/>
       <c r="B11" s="4"/>
-      <c r="C11" s="105"/>
-      <c r="D11" s="105"/>
-      <c r="E11" s="105"/>
-      <c r="F11" s="105"/>
-      <c r="G11" s="105"/>
-      <c r="H11" s="105"/>
-      <c r="I11" s="105"/>
-      <c r="J11" s="105"/>
-      <c r="K11" s="105"/>
-      <c r="L11" s="106"/>
+      <c r="C11" s="100"/>
+      <c r="D11" s="100"/>
+      <c r="E11" s="100"/>
+      <c r="F11" s="100"/>
+      <c r="G11" s="100"/>
+      <c r="H11" s="100"/>
+      <c r="I11" s="100"/>
+      <c r="J11" s="100"/>
+      <c r="K11" s="100"/>
+      <c r="L11" s="101"/>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="1"/>
       <c r="B12" s="4"/>
-      <c r="C12" s="110"/>
-      <c r="D12" s="110"/>
-      <c r="E12" s="110"/>
-      <c r="F12" s="110"/>
-      <c r="G12" s="110"/>
+      <c r="C12" s="111"/>
+      <c r="D12" s="111"/>
+      <c r="E12" s="111"/>
+      <c r="F12" s="111"/>
+      <c r="G12" s="111"/>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
@@ -2392,26 +2382,26 @@
     <row r="13" spans="1:12">
       <c r="A13" s="1"/>
       <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>6</v>
-      </c>
       <c r="D13" s="7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H13" s="5"/>
       <c r="I13" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J13" s="70"/>
       <c r="K13" s="70"/>
@@ -2462,46 +2452,46 @@
     <row r="17" spans="1:12">
       <c r="A17" s="1"/>
       <c r="B17" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="148" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="139" t="s">
+      <c r="D17" s="150"/>
+      <c r="E17" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="D17" s="141"/>
-      <c r="E17" s="45" t="s">
-        <v>10</v>
-      </c>
-      <c r="F17" s="50"/>
+      <c r="F17" s="53"/>
       <c r="G17" s="4"/>
       <c r="H17" s="8"/>
-      <c r="I17" s="45" t="s">
-        <v>11</v>
-      </c>
-      <c r="J17" s="50"/>
+      <c r="I17" s="48" t="s">
+        <v>10</v>
+      </c>
+      <c r="J17" s="53"/>
       <c r="K17" s="4"/>
-      <c r="L17" s="52"/>
+      <c r="L17" s="37"/>
     </row>
     <row r="18" spans="1:12">
       <c r="A18" s="1"/>
       <c r="B18" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="140"/>
-      <c r="D18" s="141"/>
-      <c r="E18" s="46"/>
-      <c r="F18" s="51"/>
+        <v>11</v>
+      </c>
+      <c r="C18" s="149"/>
+      <c r="D18" s="150"/>
+      <c r="E18" s="49"/>
+      <c r="F18" s="54"/>
       <c r="G18" s="4"/>
       <c r="H18" s="8"/>
-      <c r="I18" s="46"/>
-      <c r="J18" s="51"/>
+      <c r="I18" s="49"/>
+      <c r="J18" s="54"/>
       <c r="K18" s="4"/>
-      <c r="L18" s="52"/>
+      <c r="L18" s="37"/>
     </row>
     <row r="19" spans="1:12" ht="15" hidden="1" customHeight="1">
       <c r="A19" s="1"/>
       <c r="B19" s="9"/>
       <c r="C19" s="2"/>
-      <c r="D19" s="141"/>
+      <c r="D19" s="150"/>
       <c r="E19" s="9"/>
       <c r="F19" s="11"/>
       <c r="G19" s="4"/>
@@ -2514,44 +2504,44 @@
     <row r="20" spans="1:12">
       <c r="A20" s="1"/>
       <c r="B20" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" s="48"/>
-      <c r="D20" s="135"/>
-      <c r="E20" s="45" t="s">
-        <v>13</v>
-      </c>
-      <c r="F20" s="50"/>
+        <v>7</v>
+      </c>
+      <c r="C20" s="51"/>
+      <c r="D20" s="136"/>
+      <c r="E20" s="48" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" s="53"/>
       <c r="G20" s="4"/>
       <c r="H20" s="8"/>
-      <c r="I20" s="45" t="s">
-        <v>14</v>
-      </c>
-      <c r="J20" s="50"/>
+      <c r="I20" s="48" t="s">
+        <v>13</v>
+      </c>
+      <c r="J20" s="53"/>
       <c r="K20" s="4"/>
-      <c r="L20" s="52"/>
+      <c r="L20" s="37"/>
     </row>
     <row r="21" spans="1:12">
       <c r="A21" s="1"/>
       <c r="B21" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" s="49"/>
-      <c r="D21" s="135"/>
-      <c r="E21" s="47"/>
-      <c r="F21" s="49"/>
+        <v>14</v>
+      </c>
+      <c r="C21" s="52"/>
+      <c r="D21" s="136"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="52"/>
       <c r="G21" s="4"/>
       <c r="H21" s="8"/>
-      <c r="I21" s="47"/>
-      <c r="J21" s="49"/>
+      <c r="I21" s="50"/>
+      <c r="J21" s="52"/>
       <c r="K21" s="4"/>
-      <c r="L21" s="52"/>
+      <c r="L21" s="37"/>
     </row>
     <row r="22" spans="1:12">
       <c r="A22" s="1"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="52"/>
+      <c r="D22" s="37"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -2577,19 +2567,19 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="1"/>
-      <c r="B24" s="136" t="s">
-        <v>16</v>
-      </c>
-      <c r="C24" s="137"/>
-      <c r="D24" s="137"/>
-      <c r="E24" s="137"/>
-      <c r="F24" s="137"/>
-      <c r="G24" s="137"/>
-      <c r="H24" s="137"/>
-      <c r="I24" s="137"/>
-      <c r="J24" s="137"/>
-      <c r="K24" s="137"/>
-      <c r="L24" s="138"/>
+      <c r="B24" s="145" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" s="146"/>
+      <c r="D24" s="146"/>
+      <c r="E24" s="146"/>
+      <c r="F24" s="146"/>
+      <c r="G24" s="146"/>
+      <c r="H24" s="146"/>
+      <c r="I24" s="146"/>
+      <c r="J24" s="146"/>
+      <c r="K24" s="146"/>
+      <c r="L24" s="147"/>
     </row>
     <row r="25" spans="1:12">
       <c r="A25" s="1"/>
@@ -2608,56 +2598,56 @@
     <row r="26" spans="1:12">
       <c r="A26" s="1"/>
       <c r="B26" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" s="97"/>
+      <c r="D26" s="67"/>
+      <c r="E26" s="98"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="102"/>
-      <c r="D26" s="67"/>
-      <c r="E26" s="103"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="104" t="s">
-        <v>18</v>
-      </c>
-      <c r="H26" s="105"/>
-      <c r="I26" s="106"/>
-      <c r="J26" s="107"/>
-      <c r="K26" s="108"/>
-      <c r="L26" s="109"/>
+      <c r="H26" s="100"/>
+      <c r="I26" s="101"/>
+      <c r="J26" s="102"/>
+      <c r="K26" s="103"/>
+      <c r="L26" s="104"/>
     </row>
     <row r="27" spans="1:12">
       <c r="A27" s="1"/>
       <c r="B27" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="97"/>
+      <c r="D27" s="67"/>
+      <c r="E27" s="98"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="99" t="s">
         <v>19</v>
       </c>
-      <c r="C27" s="102"/>
-      <c r="D27" s="67"/>
-      <c r="E27" s="103"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="104" t="s">
-        <v>20</v>
-      </c>
-      <c r="H27" s="105"/>
-      <c r="I27" s="106"/>
-      <c r="J27" s="132"/>
-      <c r="K27" s="133"/>
-      <c r="L27" s="134"/>
+      <c r="H27" s="100"/>
+      <c r="I27" s="101"/>
+      <c r="J27" s="133"/>
+      <c r="K27" s="134"/>
+      <c r="L27" s="135"/>
     </row>
     <row r="28" spans="1:12">
       <c r="A28" s="1"/>
       <c r="B28" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="97"/>
+      <c r="D28" s="67"/>
+      <c r="E28" s="98"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="99" t="s">
         <v>21</v>
       </c>
-      <c r="C28" s="102"/>
-      <c r="D28" s="67"/>
-      <c r="E28" s="103"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="104" t="s">
-        <v>22</v>
-      </c>
-      <c r="H28" s="105"/>
-      <c r="I28" s="106"/>
-      <c r="J28" s="102"/>
+      <c r="H28" s="100"/>
+      <c r="I28" s="101"/>
+      <c r="J28" s="97"/>
       <c r="K28" s="67"/>
-      <c r="L28" s="114"/>
+      <c r="L28" s="115"/>
     </row>
     <row r="29" spans="1:12">
       <c r="A29" s="1"/>
@@ -2676,76 +2666,76 @@
     <row r="30" spans="1:12">
       <c r="A30" s="1"/>
       <c r="B30" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C30" s="119"/>
-      <c r="D30" s="119"/>
-      <c r="E30" s="119"/>
-      <c r="F30" s="119"/>
-      <c r="G30" s="119"/>
-      <c r="H30" s="119"/>
-      <c r="I30" s="119"/>
-      <c r="J30" s="119"/>
-      <c r="K30" s="119"/>
-      <c r="L30" s="120"/>
+        <v>22</v>
+      </c>
+      <c r="C30" s="131"/>
+      <c r="D30" s="131"/>
+      <c r="E30" s="131"/>
+      <c r="F30" s="131"/>
+      <c r="G30" s="131"/>
+      <c r="H30" s="131"/>
+      <c r="I30" s="131"/>
+      <c r="J30" s="131"/>
+      <c r="K30" s="131"/>
+      <c r="L30" s="132"/>
     </row>
     <row r="31" spans="1:12">
       <c r="A31" s="1"/>
-      <c r="B31" s="156"/>
-      <c r="C31" s="157"/>
-      <c r="D31" s="157"/>
-      <c r="E31" s="157"/>
-      <c r="F31" s="157"/>
-      <c r="G31" s="157"/>
-      <c r="H31" s="157"/>
-      <c r="I31" s="157"/>
-      <c r="J31" s="157"/>
-      <c r="K31" s="157"/>
-      <c r="L31" s="158"/>
+      <c r="B31" s="128"/>
+      <c r="C31" s="129"/>
+      <c r="D31" s="129"/>
+      <c r="E31" s="129"/>
+      <c r="F31" s="129"/>
+      <c r="G31" s="129"/>
+      <c r="H31" s="129"/>
+      <c r="I31" s="129"/>
+      <c r="J31" s="129"/>
+      <c r="K31" s="129"/>
+      <c r="L31" s="130"/>
     </row>
     <row r="32" spans="1:12">
       <c r="A32" s="1"/>
-      <c r="B32" s="159" t="s">
-        <v>24</v>
-      </c>
-      <c r="C32" s="119"/>
-      <c r="D32" s="119"/>
-      <c r="E32" s="119"/>
-      <c r="F32" s="119"/>
-      <c r="G32" s="119"/>
-      <c r="H32" s="119"/>
-      <c r="I32" s="119"/>
-      <c r="J32" s="119"/>
-      <c r="K32" s="119"/>
-      <c r="L32" s="120"/>
+      <c r="B32" s="137" t="s">
+        <v>23</v>
+      </c>
+      <c r="C32" s="131"/>
+      <c r="D32" s="131"/>
+      <c r="E32" s="131"/>
+      <c r="F32" s="131"/>
+      <c r="G32" s="131"/>
+      <c r="H32" s="131"/>
+      <c r="I32" s="131"/>
+      <c r="J32" s="131"/>
+      <c r="K32" s="131"/>
+      <c r="L32" s="132"/>
     </row>
     <row r="33" spans="1:12">
       <c r="A33" s="1"/>
       <c r="B33" s="77"/>
-      <c r="C33" s="121"/>
-      <c r="D33" s="121"/>
-      <c r="E33" s="121"/>
-      <c r="F33" s="121"/>
-      <c r="G33" s="121"/>
-      <c r="H33" s="121"/>
-      <c r="I33" s="121"/>
-      <c r="J33" s="121"/>
-      <c r="K33" s="121"/>
-      <c r="L33" s="121"/>
+      <c r="C33" s="138"/>
+      <c r="D33" s="138"/>
+      <c r="E33" s="138"/>
+      <c r="F33" s="138"/>
+      <c r="G33" s="138"/>
+      <c r="H33" s="138"/>
+      <c r="I33" s="138"/>
+      <c r="J33" s="138"/>
+      <c r="K33" s="138"/>
+      <c r="L33" s="138"/>
     </row>
     <row r="34" spans="1:12">
       <c r="A34" s="1"/>
-      <c r="B34" s="156"/>
-      <c r="C34" s="157"/>
-      <c r="D34" s="157"/>
-      <c r="E34" s="157"/>
-      <c r="F34" s="157"/>
-      <c r="G34" s="157"/>
-      <c r="H34" s="157"/>
-      <c r="I34" s="157"/>
-      <c r="J34" s="157"/>
-      <c r="K34" s="157"/>
-      <c r="L34" s="158"/>
+      <c r="B34" s="128"/>
+      <c r="C34" s="129"/>
+      <c r="D34" s="129"/>
+      <c r="E34" s="129"/>
+      <c r="F34" s="129"/>
+      <c r="G34" s="129"/>
+      <c r="H34" s="129"/>
+      <c r="I34" s="129"/>
+      <c r="J34" s="129"/>
+      <c r="K34" s="129"/>
+      <c r="L34" s="130"/>
     </row>
     <row r="35" spans="1:12">
       <c r="A35" s="1"/>
@@ -2763,159 +2753,159 @@
     </row>
     <row r="36" spans="1:12">
       <c r="A36" s="1"/>
-      <c r="B36" s="122" t="s">
-        <v>25</v>
-      </c>
-      <c r="C36" s="123"/>
-      <c r="D36" s="123"/>
-      <c r="E36" s="123"/>
-      <c r="F36" s="123"/>
-      <c r="G36" s="123"/>
-      <c r="H36" s="123"/>
-      <c r="I36" s="123"/>
-      <c r="J36" s="123"/>
-      <c r="K36" s="123"/>
-      <c r="L36" s="124"/>
+      <c r="B36" s="151" t="s">
+        <v>24</v>
+      </c>
+      <c r="C36" s="152"/>
+      <c r="D36" s="152"/>
+      <c r="E36" s="152"/>
+      <c r="F36" s="152"/>
+      <c r="G36" s="152"/>
+      <c r="H36" s="152"/>
+      <c r="I36" s="152"/>
+      <c r="J36" s="152"/>
+      <c r="K36" s="152"/>
+      <c r="L36" s="153"/>
     </row>
     <row r="37" spans="1:12" ht="15" customHeight="1">
       <c r="A37" s="1"/>
-      <c r="B37" s="125"/>
-      <c r="C37" s="126"/>
-      <c r="D37" s="126"/>
-      <c r="E37" s="126"/>
-      <c r="F37" s="126"/>
-      <c r="G37" s="126"/>
-      <c r="H37" s="126"/>
-      <c r="I37" s="126"/>
-      <c r="J37" s="126"/>
-      <c r="K37" s="126"/>
-      <c r="L37" s="127"/>
+      <c r="B37" s="154"/>
+      <c r="C37" s="155"/>
+      <c r="D37" s="155"/>
+      <c r="E37" s="155"/>
+      <c r="F37" s="155"/>
+      <c r="G37" s="155"/>
+      <c r="H37" s="155"/>
+      <c r="I37" s="155"/>
+      <c r="J37" s="155"/>
+      <c r="K37" s="155"/>
+      <c r="L37" s="156"/>
     </row>
     <row r="38" spans="1:12">
       <c r="A38" s="1"/>
-      <c r="B38" s="125"/>
-      <c r="C38" s="126"/>
-      <c r="D38" s="126"/>
-      <c r="E38" s="126"/>
-      <c r="F38" s="126"/>
-      <c r="G38" s="126"/>
-      <c r="H38" s="126"/>
-      <c r="I38" s="126"/>
-      <c r="J38" s="126"/>
-      <c r="K38" s="126"/>
-      <c r="L38" s="127"/>
+      <c r="B38" s="154"/>
+      <c r="C38" s="155"/>
+      <c r="D38" s="155"/>
+      <c r="E38" s="155"/>
+      <c r="F38" s="155"/>
+      <c r="G38" s="155"/>
+      <c r="H38" s="155"/>
+      <c r="I38" s="155"/>
+      <c r="J38" s="155"/>
+      <c r="K38" s="155"/>
+      <c r="L38" s="156"/>
     </row>
     <row r="39" spans="1:12">
       <c r="A39" s="1"/>
-      <c r="B39" s="125"/>
-      <c r="C39" s="126"/>
-      <c r="D39" s="126"/>
-      <c r="E39" s="126"/>
-      <c r="F39" s="126"/>
-      <c r="G39" s="126"/>
-      <c r="H39" s="126"/>
-      <c r="I39" s="126"/>
-      <c r="J39" s="126"/>
-      <c r="K39" s="126"/>
-      <c r="L39" s="127"/>
+      <c r="B39" s="154"/>
+      <c r="C39" s="155"/>
+      <c r="D39" s="155"/>
+      <c r="E39" s="155"/>
+      <c r="F39" s="155"/>
+      <c r="G39" s="155"/>
+      <c r="H39" s="155"/>
+      <c r="I39" s="155"/>
+      <c r="J39" s="155"/>
+      <c r="K39" s="155"/>
+      <c r="L39" s="156"/>
     </row>
     <row r="40" spans="1:12">
       <c r="A40" s="1"/>
-      <c r="B40" s="125"/>
-      <c r="C40" s="126"/>
-      <c r="D40" s="126"/>
-      <c r="E40" s="126"/>
-      <c r="F40" s="126"/>
-      <c r="G40" s="126"/>
-      <c r="H40" s="126"/>
-      <c r="I40" s="126"/>
-      <c r="J40" s="126"/>
-      <c r="K40" s="126"/>
-      <c r="L40" s="127"/>
+      <c r="B40" s="154"/>
+      <c r="C40" s="155"/>
+      <c r="D40" s="155"/>
+      <c r="E40" s="155"/>
+      <c r="F40" s="155"/>
+      <c r="G40" s="155"/>
+      <c r="H40" s="155"/>
+      <c r="I40" s="155"/>
+      <c r="J40" s="155"/>
+      <c r="K40" s="155"/>
+      <c r="L40" s="156"/>
     </row>
     <row r="41" spans="1:12">
       <c r="A41" s="1"/>
-      <c r="B41" s="125"/>
-      <c r="C41" s="126"/>
-      <c r="D41" s="126"/>
-      <c r="E41" s="126"/>
-      <c r="F41" s="126"/>
-      <c r="G41" s="126"/>
-      <c r="H41" s="126"/>
-      <c r="I41" s="126"/>
-      <c r="J41" s="126"/>
-      <c r="K41" s="126"/>
-      <c r="L41" s="127"/>
+      <c r="B41" s="154"/>
+      <c r="C41" s="155"/>
+      <c r="D41" s="155"/>
+      <c r="E41" s="155"/>
+      <c r="F41" s="155"/>
+      <c r="G41" s="155"/>
+      <c r="H41" s="155"/>
+      <c r="I41" s="155"/>
+      <c r="J41" s="155"/>
+      <c r="K41" s="155"/>
+      <c r="L41" s="156"/>
     </row>
     <row r="42" spans="1:12">
       <c r="A42" s="1"/>
-      <c r="B42" s="125"/>
-      <c r="C42" s="126"/>
-      <c r="D42" s="126"/>
-      <c r="E42" s="126"/>
-      <c r="F42" s="126"/>
-      <c r="G42" s="126"/>
-      <c r="H42" s="126"/>
-      <c r="I42" s="126"/>
-      <c r="J42" s="126"/>
-      <c r="K42" s="126"/>
-      <c r="L42" s="127"/>
+      <c r="B42" s="154"/>
+      <c r="C42" s="155"/>
+      <c r="D42" s="155"/>
+      <c r="E42" s="155"/>
+      <c r="F42" s="155"/>
+      <c r="G42" s="155"/>
+      <c r="H42" s="155"/>
+      <c r="I42" s="155"/>
+      <c r="J42" s="155"/>
+      <c r="K42" s="155"/>
+      <c r="L42" s="156"/>
     </row>
     <row r="43" spans="1:12">
       <c r="A43" s="1"/>
-      <c r="B43" s="125"/>
-      <c r="C43" s="126"/>
-      <c r="D43" s="126"/>
-      <c r="E43" s="126"/>
-      <c r="F43" s="126"/>
-      <c r="G43" s="126"/>
-      <c r="H43" s="126"/>
-      <c r="I43" s="126"/>
-      <c r="J43" s="126"/>
-      <c r="K43" s="126"/>
-      <c r="L43" s="127"/>
+      <c r="B43" s="154"/>
+      <c r="C43" s="155"/>
+      <c r="D43" s="155"/>
+      <c r="E43" s="155"/>
+      <c r="F43" s="155"/>
+      <c r="G43" s="155"/>
+      <c r="H43" s="155"/>
+      <c r="I43" s="155"/>
+      <c r="J43" s="155"/>
+      <c r="K43" s="155"/>
+      <c r="L43" s="156"/>
     </row>
     <row r="44" spans="1:12">
       <c r="A44" s="1"/>
-      <c r="B44" s="125"/>
-      <c r="C44" s="126"/>
-      <c r="D44" s="126"/>
-      <c r="E44" s="126"/>
-      <c r="F44" s="126"/>
-      <c r="G44" s="126"/>
-      <c r="H44" s="126"/>
-      <c r="I44" s="126"/>
-      <c r="J44" s="126"/>
-      <c r="K44" s="126"/>
-      <c r="L44" s="127"/>
+      <c r="B44" s="154"/>
+      <c r="C44" s="155"/>
+      <c r="D44" s="155"/>
+      <c r="E44" s="155"/>
+      <c r="F44" s="155"/>
+      <c r="G44" s="155"/>
+      <c r="H44" s="155"/>
+      <c r="I44" s="155"/>
+      <c r="J44" s="155"/>
+      <c r="K44" s="155"/>
+      <c r="L44" s="156"/>
     </row>
     <row r="45" spans="1:12">
       <c r="A45" s="1"/>
-      <c r="B45" s="125"/>
-      <c r="C45" s="126"/>
-      <c r="D45" s="126"/>
-      <c r="E45" s="126"/>
-      <c r="F45" s="126"/>
-      <c r="G45" s="126"/>
-      <c r="H45" s="126"/>
-      <c r="I45" s="126"/>
-      <c r="J45" s="126"/>
-      <c r="K45" s="126"/>
-      <c r="L45" s="127"/>
+      <c r="B45" s="154"/>
+      <c r="C45" s="155"/>
+      <c r="D45" s="155"/>
+      <c r="E45" s="155"/>
+      <c r="F45" s="155"/>
+      <c r="G45" s="155"/>
+      <c r="H45" s="155"/>
+      <c r="I45" s="155"/>
+      <c r="J45" s="155"/>
+      <c r="K45" s="155"/>
+      <c r="L45" s="156"/>
     </row>
     <row r="46" spans="1:12">
       <c r="A46" s="1"/>
-      <c r="B46" s="128"/>
-      <c r="C46" s="129"/>
-      <c r="D46" s="129"/>
-      <c r="E46" s="129"/>
-      <c r="F46" s="129"/>
-      <c r="G46" s="129"/>
-      <c r="H46" s="129"/>
-      <c r="I46" s="129"/>
-      <c r="J46" s="129"/>
-      <c r="K46" s="129"/>
-      <c r="L46" s="130"/>
+      <c r="B46" s="157"/>
+      <c r="C46" s="158"/>
+      <c r="D46" s="158"/>
+      <c r="E46" s="158"/>
+      <c r="F46" s="158"/>
+      <c r="G46" s="158"/>
+      <c r="H46" s="158"/>
+      <c r="I46" s="158"/>
+      <c r="J46" s="158"/>
+      <c r="K46" s="158"/>
+      <c r="L46" s="159"/>
     </row>
     <row r="47" spans="1:12">
       <c r="A47" s="1"/>
@@ -2934,18 +2924,18 @@
     <row r="48" spans="1:12">
       <c r="A48" s="1"/>
       <c r="B48" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C48" s="18"/>
       <c r="D48" s="18"/>
-      <c r="E48" s="64"/>
-      <c r="F48" s="64"/>
-      <c r="G48" s="64"/>
-      <c r="H48" s="64"/>
-      <c r="I48" s="64"/>
-      <c r="J48" s="64"/>
-      <c r="K48" s="64"/>
-      <c r="L48" s="65"/>
+      <c r="E48" s="65"/>
+      <c r="F48" s="65"/>
+      <c r="G48" s="65"/>
+      <c r="H48" s="65"/>
+      <c r="I48" s="65"/>
+      <c r="J48" s="65"/>
+      <c r="K48" s="65"/>
+      <c r="L48" s="66"/>
     </row>
     <row r="49" spans="1:12">
       <c r="A49" s="1"/>
@@ -3005,69 +2995,69 @@
     </row>
     <row r="53" spans="1:12" ht="30" customHeight="1">
       <c r="A53" s="1"/>
-      <c r="B53" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="C53" s="131"/>
-      <c r="D53" s="131"/>
-      <c r="E53" s="131"/>
-      <c r="F53" s="131"/>
-      <c r="G53" s="131"/>
-      <c r="H53" s="131"/>
-      <c r="I53" s="131"/>
-      <c r="J53" s="131"/>
-      <c r="K53" s="131"/>
-      <c r="L53" s="131"/>
+      <c r="B53" s="105" t="s">
+        <v>26</v>
+      </c>
+      <c r="C53" s="105"/>
+      <c r="D53" s="105"/>
+      <c r="E53" s="105"/>
+      <c r="F53" s="105"/>
+      <c r="G53" s="105"/>
+      <c r="H53" s="105"/>
+      <c r="I53" s="105"/>
+      <c r="J53" s="105"/>
+      <c r="K53" s="105"/>
+      <c r="L53" s="105"/>
     </row>
     <row r="54" spans="1:12">
       <c r="A54" s="1"/>
-      <c r="B54" s="63" t="s">
+      <c r="B54" s="64" t="s">
+        <v>27</v>
+      </c>
+      <c r="C54" s="66"/>
+      <c r="D54" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="C54" s="65"/>
-      <c r="D54" s="63" t="s">
+      <c r="E54" s="65"/>
+      <c r="F54" s="66"/>
+      <c r="G54" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="E54" s="64"/>
-      <c r="F54" s="65"/>
-      <c r="G54" s="63" t="s">
+      <c r="H54" s="65"/>
+      <c r="I54" s="65"/>
+      <c r="J54" s="66"/>
+      <c r="K54" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="H54" s="64"/>
-      <c r="I54" s="64"/>
-      <c r="J54" s="65"/>
-      <c r="K54" s="63" t="s">
-        <v>31</v>
-      </c>
-      <c r="L54" s="65"/>
+      <c r="L54" s="66"/>
     </row>
     <row r="55" spans="1:12">
       <c r="A55" s="1"/>
-      <c r="B55" s="63"/>
-      <c r="C55" s="65"/>
-      <c r="D55" s="63"/>
-      <c r="E55" s="64"/>
-      <c r="F55" s="65"/>
-      <c r="G55" s="153"/>
-      <c r="H55" s="154"/>
-      <c r="I55" s="154"/>
-      <c r="J55" s="155"/>
-      <c r="K55" s="153"/>
-      <c r="L55" s="155"/>
+      <c r="B55" s="64"/>
+      <c r="C55" s="66"/>
+      <c r="D55" s="64"/>
+      <c r="E55" s="65"/>
+      <c r="F55" s="66"/>
+      <c r="G55" s="125"/>
+      <c r="H55" s="126"/>
+      <c r="I55" s="126"/>
+      <c r="J55" s="127"/>
+      <c r="K55" s="125"/>
+      <c r="L55" s="127"/>
     </row>
     <row r="56" spans="1:12">
       <c r="A56" s="1"/>
-      <c r="B56" s="63"/>
-      <c r="C56" s="65"/>
-      <c r="D56" s="63"/>
-      <c r="E56" s="64"/>
-      <c r="F56" s="65"/>
-      <c r="G56" s="153"/>
-      <c r="H56" s="154"/>
-      <c r="I56" s="154"/>
-      <c r="J56" s="155"/>
-      <c r="K56" s="153"/>
-      <c r="L56" s="155"/>
+      <c r="B56" s="64"/>
+      <c r="C56" s="66"/>
+      <c r="D56" s="64"/>
+      <c r="E56" s="65"/>
+      <c r="F56" s="66"/>
+      <c r="G56" s="125"/>
+      <c r="H56" s="126"/>
+      <c r="I56" s="126"/>
+      <c r="J56" s="127"/>
+      <c r="K56" s="125"/>
+      <c r="L56" s="127"/>
     </row>
     <row r="57" spans="1:12">
       <c r="A57" s="1"/>
@@ -3106,49 +3096,49 @@
       <c r="H59" s="95"/>
       <c r="I59" s="95"/>
       <c r="J59" s="96"/>
-      <c r="K59" s="111"/>
-      <c r="L59" s="112"/>
-    </row>
-    <row r="60" spans="1:12" s="34" customFormat="1" ht="90.75" customHeight="1">
+      <c r="K59" s="112"/>
+      <c r="L59" s="113"/>
+    </row>
+    <row r="60" spans="1:12" s="34" customFormat="1" ht="95.25" customHeight="1">
       <c r="A60" s="33"/>
-      <c r="B60" s="37" t="s">
+      <c r="B60" s="40" t="s">
+        <v>31</v>
+      </c>
+      <c r="C60" s="42"/>
+      <c r="D60" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C60" s="39"/>
-      <c r="D60" s="37" t="s">
+      <c r="E60" s="41"/>
+      <c r="F60" s="42"/>
+      <c r="G60" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="E60" s="38"/>
-      <c r="F60" s="39"/>
-      <c r="G60" s="37" t="s">
+      <c r="H60" s="41"/>
+      <c r="I60" s="41"/>
+      <c r="J60" s="42"/>
+      <c r="K60" s="118" t="s">
         <v>34</v>
       </c>
-      <c r="H60" s="38"/>
-      <c r="I60" s="38"/>
-      <c r="J60" s="39"/>
-      <c r="K60" s="117" t="s">
-        <v>35</v>
-      </c>
-      <c r="L60" s="118"/>
-    </row>
-    <row r="61" spans="1:12" ht="15" customHeight="1"/>
-    <row r="62" spans="1:12" ht="27" customHeight="1"/>
-    <row r="63" spans="1:12" ht="27" customHeight="1"/>
-    <row r="64" spans="1:12" ht="33" customHeight="1"/>
-    <row r="65" spans="1:12" ht="15" customHeight="1"/>
-    <row r="66" spans="1:12" ht="33" customHeight="1"/>
-    <row r="67" spans="1:12" ht="15" customHeight="1"/>
+      <c r="L60" s="119"/>
+    </row>
+    <row r="61" spans="1:12" ht="30" customHeight="1"/>
+    <row r="62" spans="1:12" ht="30" customHeight="1"/>
+    <row r="63" spans="1:12" ht="30" customHeight="1"/>
+    <row r="64" spans="1:12" ht="15" customHeight="1"/>
+    <row r="65" spans="1:12" ht="33" customHeight="1"/>
+    <row r="66" spans="1:12" ht="15" customHeight="1"/>
+    <row r="67" spans="1:12" ht="33" customHeight="1"/>
     <row r="68" spans="1:12">
       <c r="A68" s="1"/>
       <c r="B68" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C68" s="2"/>
-      <c r="D68" s="43" t="s">
-        <v>1</v>
+      <c r="D68" s="46" t="s">
+        <v>35</v>
       </c>
       <c r="E68" s="72"/>
-      <c r="F68" s="44"/>
+      <c r="F68" s="47"/>
       <c r="G68" s="2"/>
       <c r="H68" s="2"/>
       <c r="I68" s="2"/>
@@ -3159,12 +3149,12 @@
     <row r="69" spans="1:12">
       <c r="A69" s="1"/>
       <c r="B69" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C69" s="2"/>
-      <c r="D69" s="113"/>
-      <c r="E69" s="113"/>
-      <c r="F69" s="113"/>
+      <c r="D69" s="114"/>
+      <c r="E69" s="114"/>
+      <c r="F69" s="114"/>
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
       <c r="I69" s="2"/>
@@ -3189,7 +3179,7 @@
     <row r="71" spans="1:12">
       <c r="A71" s="1"/>
       <c r="B71" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C71" s="67"/>
       <c r="D71" s="67"/>
@@ -3200,26 +3190,26 @@
       <c r="I71" s="67"/>
       <c r="J71" s="67"/>
       <c r="K71" s="67"/>
-      <c r="L71" s="114"/>
+      <c r="L71" s="115"/>
     </row>
     <row r="72" spans="1:12">
       <c r="A72" s="1"/>
       <c r="B72" s="4"/>
-      <c r="C72" s="115"/>
-      <c r="D72" s="115"/>
-      <c r="E72" s="115"/>
-      <c r="F72" s="115"/>
-      <c r="G72" s="115"/>
-      <c r="H72" s="115"/>
-      <c r="I72" s="115"/>
-      <c r="J72" s="115"/>
-      <c r="K72" s="115"/>
-      <c r="L72" s="116"/>
+      <c r="C72" s="116"/>
+      <c r="D72" s="116"/>
+      <c r="E72" s="116"/>
+      <c r="F72" s="116"/>
+      <c r="G72" s="116"/>
+      <c r="H72" s="116"/>
+      <c r="I72" s="116"/>
+      <c r="J72" s="116"/>
+      <c r="K72" s="116"/>
+      <c r="L72" s="117"/>
     </row>
     <row r="73" spans="1:12">
       <c r="A73" s="1"/>
       <c r="B73" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C73" s="70"/>
       <c r="D73" s="70"/>
@@ -3235,25 +3225,25 @@
     <row r="74" spans="1:12">
       <c r="A74" s="1"/>
       <c r="B74" s="4"/>
-      <c r="C74" s="105"/>
-      <c r="D74" s="105"/>
-      <c r="E74" s="105"/>
-      <c r="F74" s="105"/>
-      <c r="G74" s="105"/>
-      <c r="H74" s="105"/>
-      <c r="I74" s="105"/>
-      <c r="J74" s="105"/>
-      <c r="K74" s="105"/>
-      <c r="L74" s="106"/>
+      <c r="C74" s="100"/>
+      <c r="D74" s="100"/>
+      <c r="E74" s="100"/>
+      <c r="F74" s="100"/>
+      <c r="G74" s="100"/>
+      <c r="H74" s="100"/>
+      <c r="I74" s="100"/>
+      <c r="J74" s="100"/>
+      <c r="K74" s="100"/>
+      <c r="L74" s="101"/>
     </row>
     <row r="75" spans="1:12">
       <c r="A75" s="1"/>
       <c r="B75" s="4"/>
-      <c r="C75" s="110"/>
-      <c r="D75" s="110"/>
-      <c r="E75" s="110"/>
-      <c r="F75" s="110"/>
-      <c r="G75" s="110"/>
+      <c r="C75" s="111"/>
+      <c r="D75" s="111"/>
+      <c r="E75" s="111"/>
+      <c r="F75" s="111"/>
+      <c r="G75" s="111"/>
       <c r="H75" s="5"/>
       <c r="I75" s="5"/>
       <c r="J75" s="5"/>
@@ -3263,7 +3253,7 @@
     <row r="76" spans="1:12">
       <c r="A76" s="1"/>
       <c r="B76" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C76" s="7"/>
       <c r="D76" s="26"/>
@@ -3272,7 +3262,7 @@
       <c r="G76" s="27"/>
       <c r="H76" s="5"/>
       <c r="I76" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J76" s="70"/>
       <c r="K76" s="70"/>
@@ -3322,19 +3312,19 @@
     </row>
     <row r="80" spans="1:12">
       <c r="A80" s="1"/>
-      <c r="B80" s="63" t="s">
-        <v>16</v>
-      </c>
-      <c r="C80" s="64"/>
-      <c r="D80" s="64"/>
-      <c r="E80" s="64"/>
-      <c r="F80" s="64"/>
-      <c r="G80" s="64"/>
-      <c r="H80" s="64"/>
-      <c r="I80" s="64"/>
-      <c r="J80" s="64"/>
-      <c r="K80" s="64"/>
-      <c r="L80" s="65"/>
+      <c r="B80" s="64" t="s">
+        <v>15</v>
+      </c>
+      <c r="C80" s="65"/>
+      <c r="D80" s="65"/>
+      <c r="E80" s="65"/>
+      <c r="F80" s="65"/>
+      <c r="G80" s="65"/>
+      <c r="H80" s="65"/>
+      <c r="I80" s="65"/>
+      <c r="J80" s="65"/>
+      <c r="K80" s="65"/>
+      <c r="L80" s="66"/>
     </row>
     <row r="81" spans="1:12">
       <c r="A81" s="1"/>
@@ -3353,56 +3343,56 @@
     <row r="82" spans="1:12">
       <c r="A82" s="1"/>
       <c r="B82" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C82" s="97"/>
+      <c r="D82" s="67"/>
+      <c r="E82" s="98"/>
+      <c r="F82" s="13"/>
+      <c r="G82" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="C82" s="102"/>
-      <c r="D82" s="67"/>
-      <c r="E82" s="103"/>
-      <c r="F82" s="13"/>
-      <c r="G82" s="104" t="s">
-        <v>18</v>
-      </c>
-      <c r="H82" s="105"/>
-      <c r="I82" s="106"/>
-      <c r="J82" s="107"/>
-      <c r="K82" s="108"/>
-      <c r="L82" s="109"/>
+      <c r="H82" s="100"/>
+      <c r="I82" s="101"/>
+      <c r="J82" s="102"/>
+      <c r="K82" s="103"/>
+      <c r="L82" s="104"/>
     </row>
     <row r="83" spans="1:12">
       <c r="A83" s="1"/>
       <c r="B83" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C83" s="97"/>
+      <c r="D83" s="67"/>
+      <c r="E83" s="98"/>
+      <c r="F83" s="2"/>
+      <c r="G83" s="99" t="s">
         <v>19</v>
       </c>
-      <c r="C83" s="102"/>
-      <c r="D83" s="67"/>
-      <c r="E83" s="103"/>
-      <c r="F83" s="2"/>
-      <c r="G83" s="104" t="s">
-        <v>20</v>
-      </c>
-      <c r="H83" s="105"/>
-      <c r="I83" s="106"/>
-      <c r="J83" s="107"/>
-      <c r="K83" s="108"/>
-      <c r="L83" s="109"/>
+      <c r="H83" s="100"/>
+      <c r="I83" s="101"/>
+      <c r="J83" s="102"/>
+      <c r="K83" s="103"/>
+      <c r="L83" s="104"/>
     </row>
     <row r="84" spans="1:12">
       <c r="A84" s="1"/>
       <c r="B84" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C84" s="97"/>
+      <c r="D84" s="67"/>
+      <c r="E84" s="98"/>
+      <c r="F84" s="8"/>
+      <c r="G84" s="99" t="s">
         <v>21</v>
       </c>
-      <c r="C84" s="102"/>
-      <c r="D84" s="67"/>
-      <c r="E84" s="103"/>
-      <c r="F84" s="8"/>
-      <c r="G84" s="104" t="s">
-        <v>22</v>
-      </c>
-      <c r="H84" s="105"/>
-      <c r="I84" s="106"/>
-      <c r="J84" s="107"/>
-      <c r="K84" s="108"/>
-      <c r="L84" s="109"/>
+      <c r="H84" s="100"/>
+      <c r="I84" s="101"/>
+      <c r="J84" s="102"/>
+      <c r="K84" s="103"/>
+      <c r="L84" s="104"/>
     </row>
     <row r="85" spans="1:12">
       <c r="A85" s="1"/>
@@ -3434,37 +3424,37 @@
     </row>
     <row r="87" spans="1:12">
       <c r="A87" s="1"/>
-      <c r="B87" s="63" t="s">
+      <c r="B87" s="64" t="s">
         <v>36</v>
       </c>
-      <c r="C87" s="64"/>
-      <c r="D87" s="64"/>
-      <c r="E87" s="64"/>
-      <c r="F87" s="64"/>
-      <c r="G87" s="64"/>
-      <c r="H87" s="64"/>
-      <c r="I87" s="64"/>
-      <c r="J87" s="65"/>
-      <c r="K87" s="63" t="s">
+      <c r="C87" s="65"/>
+      <c r="D87" s="65"/>
+      <c r="E87" s="65"/>
+      <c r="F87" s="65"/>
+      <c r="G87" s="65"/>
+      <c r="H87" s="65"/>
+      <c r="I87" s="65"/>
+      <c r="J87" s="66"/>
+      <c r="K87" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="L87" s="65"/>
+      <c r="L87" s="66"/>
     </row>
     <row r="88" spans="1:12">
       <c r="A88" s="1"/>
-      <c r="B88" s="97" t="s">
+      <c r="B88" s="106" t="s">
         <v>38</v>
       </c>
-      <c r="C88" s="98"/>
-      <c r="D88" s="98"/>
-      <c r="E88" s="98"/>
-      <c r="F88" s="98"/>
-      <c r="G88" s="98"/>
-      <c r="H88" s="98"/>
-      <c r="I88" s="98"/>
-      <c r="J88" s="99"/>
-      <c r="K88" s="100"/>
-      <c r="L88" s="101"/>
+      <c r="C88" s="107"/>
+      <c r="D88" s="107"/>
+      <c r="E88" s="107"/>
+      <c r="F88" s="107"/>
+      <c r="G88" s="107"/>
+      <c r="H88" s="107"/>
+      <c r="I88" s="107"/>
+      <c r="J88" s="108"/>
+      <c r="K88" s="109"/>
+      <c r="L88" s="110"/>
     </row>
     <row r="89" spans="1:12">
       <c r="A89" s="1"/>
@@ -3900,59 +3890,59 @@
     </row>
     <row r="116" spans="1:12">
       <c r="A116" s="1"/>
-      <c r="B116" s="142"/>
-      <c r="C116" s="143"/>
-      <c r="D116" s="143"/>
-      <c r="E116" s="143"/>
-      <c r="F116" s="143"/>
-      <c r="G116" s="143"/>
-      <c r="H116" s="143"/>
-      <c r="I116" s="143"/>
-      <c r="J116" s="144"/>
-      <c r="K116" s="142"/>
-      <c r="L116" s="144"/>
+      <c r="B116" s="139"/>
+      <c r="C116" s="140"/>
+      <c r="D116" s="140"/>
+      <c r="E116" s="140"/>
+      <c r="F116" s="140"/>
+      <c r="G116" s="140"/>
+      <c r="H116" s="140"/>
+      <c r="I116" s="140"/>
+      <c r="J116" s="141"/>
+      <c r="K116" s="139"/>
+      <c r="L116" s="141"/>
     </row>
     <row r="117" spans="1:12">
       <c r="A117" s="1"/>
-      <c r="B117" s="135"/>
-      <c r="C117" s="52"/>
-      <c r="D117" s="52"/>
-      <c r="E117" s="52"/>
-      <c r="F117" s="52"/>
-      <c r="G117" s="52"/>
-      <c r="H117" s="52"/>
-      <c r="I117" s="52"/>
-      <c r="J117" s="145"/>
-      <c r="K117" s="135"/>
-      <c r="L117" s="145"/>
+      <c r="B117" s="136"/>
+      <c r="C117" s="37"/>
+      <c r="D117" s="37"/>
+      <c r="E117" s="37"/>
+      <c r="F117" s="37"/>
+      <c r="G117" s="37"/>
+      <c r="H117" s="37"/>
+      <c r="I117" s="37"/>
+      <c r="J117" s="142"/>
+      <c r="K117" s="136"/>
+      <c r="L117" s="142"/>
     </row>
     <row r="118" spans="1:12">
       <c r="A118" s="1"/>
-      <c r="B118" s="135"/>
-      <c r="C118" s="52"/>
-      <c r="D118" s="52"/>
-      <c r="E118" s="52"/>
-      <c r="F118" s="52"/>
-      <c r="G118" s="52"/>
-      <c r="H118" s="52"/>
-      <c r="I118" s="52"/>
-      <c r="J118" s="145"/>
-      <c r="K118" s="135"/>
-      <c r="L118" s="145"/>
+      <c r="B118" s="136"/>
+      <c r="C118" s="37"/>
+      <c r="D118" s="37"/>
+      <c r="E118" s="37"/>
+      <c r="F118" s="37"/>
+      <c r="G118" s="37"/>
+      <c r="H118" s="37"/>
+      <c r="I118" s="37"/>
+      <c r="J118" s="142"/>
+      <c r="K118" s="136"/>
+      <c r="L118" s="142"/>
     </row>
     <row r="119" spans="1:12" ht="45" customHeight="1">
       <c r="A119" s="1"/>
-      <c r="B119" s="146"/>
-      <c r="C119" s="131"/>
-      <c r="D119" s="131"/>
-      <c r="E119" s="131"/>
-      <c r="F119" s="131"/>
-      <c r="G119" s="131"/>
-      <c r="H119" s="131"/>
-      <c r="I119" s="131"/>
-      <c r="J119" s="147"/>
-      <c r="K119" s="146"/>
-      <c r="L119" s="147"/>
+      <c r="B119" s="143"/>
+      <c r="C119" s="105"/>
+      <c r="D119" s="105"/>
+      <c r="E119" s="105"/>
+      <c r="F119" s="105"/>
+      <c r="G119" s="105"/>
+      <c r="H119" s="105"/>
+      <c r="I119" s="105"/>
+      <c r="J119" s="144"/>
+      <c r="K119" s="143"/>
+      <c r="L119" s="144"/>
     </row>
     <row r="120" spans="1:12">
       <c r="A120" s="1"/>
@@ -4008,47 +3998,48 @@
       <c r="K123" s="94"/>
       <c r="L123" s="96"/>
     </row>
-    <row r="124" spans="1:12" s="31" customFormat="1" ht="47.25" customHeight="1">
+    <row r="124" spans="1:12" s="31" customFormat="1" ht="50.25" customHeight="1">
       <c r="A124" s="25"/>
-      <c r="B124" s="35" t="s">
+      <c r="B124" s="38" t="s">
+        <v>31</v>
+      </c>
+      <c r="C124" s="39"/>
+      <c r="D124" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C124" s="36"/>
-      <c r="D124" s="37" t="s">
+      <c r="E124" s="41"/>
+      <c r="F124" s="42"/>
+      <c r="G124" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="E124" s="38"/>
-      <c r="F124" s="39"/>
-      <c r="G124" s="37" t="s">
+      <c r="H124" s="41"/>
+      <c r="I124" s="41"/>
+      <c r="J124" s="42"/>
+      <c r="K124" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="H124" s="38"/>
-      <c r="I124" s="38"/>
-      <c r="J124" s="39"/>
-      <c r="K124" s="37" t="s">
-        <v>35</v>
-      </c>
-      <c r="L124" s="39"/>
-    </row>
-    <row r="126" spans="1:12" ht="27" customHeight="1"/>
-    <row r="127" spans="1:12" ht="27" customHeight="1"/>
-    <row r="128" spans="1:12" ht="33" customHeight="1"/>
-    <row r="129" spans="1:12" ht="15" customHeight="1"/>
-    <row r="130" spans="1:12" ht="33" customHeight="1"/>
-    <row r="131" spans="1:12" ht="15" customHeight="1"/>
+      <c r="L124" s="42"/>
+    </row>
+    <row r="125" spans="1:12" ht="30" customHeight="1"/>
+    <row r="126" spans="1:12" ht="30" customHeight="1"/>
+    <row r="127" spans="1:12" ht="30" customHeight="1"/>
+    <row r="128" spans="1:12" ht="15" customHeight="1"/>
+    <row r="129" spans="1:12" ht="33" customHeight="1"/>
+    <row r="130" spans="1:12" ht="15" customHeight="1"/>
+    <row r="131" spans="1:12" ht="33" customHeight="1"/>
     <row r="132" spans="1:12">
       <c r="A132" s="1"/>
       <c r="B132" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C132" s="2"/>
-      <c r="D132" s="43" t="str">
+      <c r="D132" s="46" t="str">
         <f>D68</f>
         <v>MHOS-SSM-EL-0001</v>
       </c>
       <c r="E132" s="72"/>
       <c r="F132" s="72"/>
-      <c r="G132" s="44"/>
+      <c r="G132" s="47"/>
       <c r="H132" s="2"/>
       <c r="I132" s="2"/>
       <c r="J132" s="2"/>
@@ -4058,7 +4049,7 @@
     <row r="133" spans="1:12">
       <c r="A133" s="1"/>
       <c r="B133" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C133" s="2"/>
       <c r="D133" s="73"/>
@@ -4088,7 +4079,7 @@
     <row r="135" spans="1:12">
       <c r="A135" s="1"/>
       <c r="B135" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C135" s="67"/>
       <c r="D135" s="67"/>
@@ -4118,7 +4109,7 @@
     <row r="137" spans="1:12">
       <c r="A137" s="1"/>
       <c r="B137" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C137" s="70"/>
       <c r="D137" s="70"/>
@@ -4127,7 +4118,7 @@
       <c r="G137" s="70"/>
       <c r="H137" s="5"/>
       <c r="I137" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J137" s="70"/>
       <c r="K137" s="70"/>
@@ -4163,19 +4154,19 @@
     </row>
     <row r="140" spans="1:12">
       <c r="A140" s="1"/>
-      <c r="B140" s="63" t="s">
+      <c r="B140" s="64" t="s">
         <v>66</v>
       </c>
-      <c r="C140" s="64"/>
-      <c r="D140" s="64"/>
-      <c r="E140" s="64"/>
-      <c r="F140" s="64"/>
-      <c r="G140" s="64"/>
-      <c r="H140" s="64"/>
-      <c r="I140" s="64"/>
-      <c r="J140" s="64"/>
-      <c r="K140" s="64"/>
-      <c r="L140" s="65"/>
+      <c r="C140" s="65"/>
+      <c r="D140" s="65"/>
+      <c r="E140" s="65"/>
+      <c r="F140" s="65"/>
+      <c r="G140" s="65"/>
+      <c r="H140" s="65"/>
+      <c r="I140" s="65"/>
+      <c r="J140" s="65"/>
+      <c r="K140" s="65"/>
+      <c r="L140" s="66"/>
     </row>
     <row r="141" spans="1:12">
       <c r="A141" s="1"/>
@@ -4207,115 +4198,115 @@
     </row>
     <row r="143" spans="1:12">
       <c r="A143" s="1"/>
-      <c r="B143" s="66"/>
-      <c r="C143" s="66"/>
-      <c r="D143" s="66"/>
-      <c r="E143" s="66"/>
-      <c r="F143" s="66"/>
-      <c r="G143" s="66"/>
-      <c r="H143" s="66"/>
-      <c r="I143" s="66"/>
-      <c r="J143" s="66"/>
-      <c r="K143" s="66"/>
-      <c r="L143" s="66"/>
+      <c r="B143" s="29"/>
+      <c r="C143" s="29"/>
+      <c r="D143" s="29"/>
+      <c r="E143" s="29"/>
+      <c r="F143" s="29"/>
+      <c r="G143" s="29"/>
+      <c r="H143" s="29"/>
+      <c r="I143" s="29"/>
+      <c r="J143" s="29"/>
+      <c r="K143" s="29"/>
+      <c r="L143" s="29"/>
     </row>
     <row r="144" spans="1:12">
       <c r="A144" s="1"/>
-      <c r="B144" s="66"/>
-      <c r="C144" s="66"/>
-      <c r="D144" s="66"/>
-      <c r="E144" s="66"/>
-      <c r="F144" s="66"/>
-      <c r="G144" s="66"/>
-      <c r="H144" s="66"/>
-      <c r="I144" s="66"/>
-      <c r="J144" s="66"/>
-      <c r="K144" s="66"/>
-      <c r="L144" s="66"/>
+      <c r="B144" s="29"/>
+      <c r="C144" s="29"/>
+      <c r="D144" s="29"/>
+      <c r="E144" s="29"/>
+      <c r="F144" s="29"/>
+      <c r="G144" s="29"/>
+      <c r="H144" s="29"/>
+      <c r="I144" s="29"/>
+      <c r="J144" s="29"/>
+      <c r="K144" s="29"/>
+      <c r="L144" s="29"/>
     </row>
     <row r="145" spans="1:12">
       <c r="A145" s="1"/>
-      <c r="B145" s="66"/>
-      <c r="C145" s="66"/>
-      <c r="D145" s="66"/>
-      <c r="E145" s="66"/>
-      <c r="F145" s="66"/>
-      <c r="G145" s="66"/>
-      <c r="H145" s="66"/>
-      <c r="I145" s="66"/>
-      <c r="J145" s="66"/>
-      <c r="K145" s="66"/>
-      <c r="L145" s="66"/>
+      <c r="B145" s="29"/>
+      <c r="C145" s="29"/>
+      <c r="D145" s="29"/>
+      <c r="E145" s="29"/>
+      <c r="F145" s="29"/>
+      <c r="G145" s="29"/>
+      <c r="H145" s="29"/>
+      <c r="I145" s="29"/>
+      <c r="J145" s="29"/>
+      <c r="K145" s="29"/>
+      <c r="L145" s="29"/>
     </row>
     <row r="146" spans="1:12">
       <c r="A146" s="1"/>
-      <c r="B146" s="66"/>
-      <c r="C146" s="66"/>
-      <c r="D146" s="66"/>
-      <c r="E146" s="66"/>
-      <c r="F146" s="66"/>
-      <c r="G146" s="66"/>
-      <c r="H146" s="66"/>
-      <c r="I146" s="66"/>
-      <c r="J146" s="66"/>
-      <c r="K146" s="66"/>
-      <c r="L146" s="66"/>
+      <c r="B146" s="29"/>
+      <c r="C146" s="29"/>
+      <c r="D146" s="29"/>
+      <c r="E146" s="29"/>
+      <c r="F146" s="29"/>
+      <c r="G146" s="29"/>
+      <c r="H146" s="29"/>
+      <c r="I146" s="29"/>
+      <c r="J146" s="29"/>
+      <c r="K146" s="29"/>
+      <c r="L146" s="29"/>
     </row>
     <row r="147" spans="1:12">
       <c r="A147" s="1"/>
-      <c r="B147" s="66"/>
-      <c r="C147" s="66"/>
-      <c r="D147" s="66"/>
-      <c r="E147" s="66"/>
-      <c r="F147" s="66"/>
-      <c r="G147" s="66"/>
-      <c r="H147" s="66"/>
-      <c r="I147" s="66"/>
-      <c r="J147" s="66"/>
-      <c r="K147" s="66"/>
-      <c r="L147" s="66"/>
+      <c r="B147" s="29"/>
+      <c r="C147" s="29"/>
+      <c r="D147" s="29"/>
+      <c r="E147" s="29"/>
+      <c r="F147" s="29"/>
+      <c r="G147" s="29"/>
+      <c r="H147" s="29"/>
+      <c r="I147" s="29"/>
+      <c r="J147" s="29"/>
+      <c r="K147" s="29"/>
+      <c r="L147" s="29"/>
     </row>
     <row r="148" spans="1:12">
       <c r="A148" s="1"/>
-      <c r="B148" s="66"/>
-      <c r="C148" s="66"/>
-      <c r="D148" s="66"/>
-      <c r="E148" s="66"/>
-      <c r="F148" s="66"/>
-      <c r="G148" s="66"/>
-      <c r="H148" s="66"/>
-      <c r="I148" s="66"/>
-      <c r="J148" s="66"/>
-      <c r="K148" s="66"/>
-      <c r="L148" s="66"/>
+      <c r="B148" s="29"/>
+      <c r="C148" s="29"/>
+      <c r="D148" s="29"/>
+      <c r="E148" s="29"/>
+      <c r="F148" s="29"/>
+      <c r="G148" s="29"/>
+      <c r="H148" s="29"/>
+      <c r="I148" s="29"/>
+      <c r="J148" s="29"/>
+      <c r="K148" s="29"/>
+      <c r="L148" s="29"/>
     </row>
     <row r="149" spans="1:12">
       <c r="A149" s="1"/>
-      <c r="B149" s="66"/>
-      <c r="C149" s="66"/>
-      <c r="D149" s="66"/>
-      <c r="E149" s="66"/>
-      <c r="F149" s="66"/>
-      <c r="G149" s="66"/>
-      <c r="H149" s="66"/>
-      <c r="I149" s="66"/>
-      <c r="J149" s="66"/>
-      <c r="K149" s="66"/>
-      <c r="L149" s="66"/>
+      <c r="B149" s="29"/>
+      <c r="C149" s="29"/>
+      <c r="D149" s="29"/>
+      <c r="E149" s="29"/>
+      <c r="F149" s="29"/>
+      <c r="G149" s="29"/>
+      <c r="H149" s="29"/>
+      <c r="I149" s="29"/>
+      <c r="J149" s="29"/>
+      <c r="K149" s="29"/>
+      <c r="L149" s="29"/>
     </row>
     <row r="150" spans="1:12" ht="31.5" customHeight="1">
       <c r="A150" s="1"/>
-      <c r="B150" s="66"/>
-      <c r="C150" s="66"/>
-      <c r="D150" s="66"/>
-      <c r="E150" s="66"/>
-      <c r="F150" s="66"/>
-      <c r="G150" s="66"/>
-      <c r="H150" s="66"/>
-      <c r="I150" s="66"/>
-      <c r="J150" s="66"/>
-      <c r="K150" s="66"/>
-      <c r="L150" s="66"/>
+      <c r="B150" s="29"/>
+      <c r="C150" s="29"/>
+      <c r="D150" s="29"/>
+      <c r="E150" s="29"/>
+      <c r="F150" s="29"/>
+      <c r="G150" s="29"/>
+      <c r="H150" s="29"/>
+      <c r="I150" s="29"/>
+      <c r="J150" s="29"/>
+      <c r="K150" s="29"/>
+      <c r="L150" s="29"/>
     </row>
     <row r="151" spans="1:12">
       <c r="A151" s="1"/>
@@ -4333,21 +4324,21 @@
     </row>
     <row r="152" spans="1:12">
       <c r="A152" s="1"/>
-      <c r="B152" s="52" t="s">
+      <c r="B152" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="C152" s="52"/>
-      <c r="D152" s="2"/>
-      <c r="E152" s="2"/>
+      <c r="C152" s="37"/>
+      <c r="D152" s="37"/>
+      <c r="E152" s="37"/>
       <c r="F152" s="2"/>
-      <c r="G152" s="2"/>
-      <c r="H152" s="2"/>
-      <c r="I152" s="52" t="s">
+      <c r="G152" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="J152" s="52"/>
-      <c r="K152" s="2"/>
-      <c r="L152" s="2"/>
+      <c r="H152" s="37"/>
+      <c r="I152" s="37"/>
+      <c r="J152" s="37"/>
+      <c r="K152" s="37"/>
+      <c r="L152" s="37"/>
     </row>
     <row r="153" spans="1:12">
       <c r="A153" s="1"/>
@@ -4395,117 +4386,117 @@
     </row>
     <row r="156" spans="1:12">
       <c r="A156" s="1"/>
-      <c r="B156" s="62"/>
-      <c r="C156" s="62"/>
-      <c r="D156" s="52"/>
-      <c r="E156" s="52"/>
-      <c r="F156" s="52"/>
-      <c r="G156" s="2"/>
-      <c r="H156" s="52"/>
-      <c r="I156" s="52"/>
-      <c r="J156" s="52"/>
-      <c r="K156" s="52"/>
-      <c r="L156" s="52"/>
+      <c r="B156" s="30"/>
+      <c r="C156" s="30"/>
+      <c r="D156" s="30"/>
+      <c r="E156" s="30"/>
+      <c r="F156" s="30"/>
+      <c r="G156" s="30"/>
+      <c r="H156" s="30"/>
+      <c r="I156" s="30"/>
+      <c r="J156" s="30"/>
+      <c r="K156" s="30"/>
+      <c r="L156" s="30"/>
     </row>
     <row r="157" spans="1:12">
       <c r="A157" s="1"/>
-      <c r="B157" s="62"/>
-      <c r="C157" s="62"/>
-      <c r="D157" s="52"/>
-      <c r="E157" s="52"/>
-      <c r="F157" s="52"/>
-      <c r="G157" s="2"/>
-      <c r="H157" s="52"/>
-      <c r="I157" s="52"/>
-      <c r="J157" s="52"/>
-      <c r="K157" s="52"/>
-      <c r="L157" s="52"/>
+      <c r="B157" s="30"/>
+      <c r="C157" s="30"/>
+      <c r="D157" s="30"/>
+      <c r="E157" s="30"/>
+      <c r="F157" s="30"/>
+      <c r="G157" s="30"/>
+      <c r="H157" s="30"/>
+      <c r="I157" s="30"/>
+      <c r="J157" s="30"/>
+      <c r="K157" s="30"/>
+      <c r="L157" s="30"/>
     </row>
     <row r="158" spans="1:12">
       <c r="A158" s="1"/>
-      <c r="B158" s="62"/>
-      <c r="C158" s="62"/>
-      <c r="D158" s="52"/>
-      <c r="E158" s="52"/>
-      <c r="F158" s="52"/>
-      <c r="G158" s="2"/>
-      <c r="H158" s="52"/>
-      <c r="I158" s="52"/>
-      <c r="J158" s="52"/>
-      <c r="K158" s="52"/>
-      <c r="L158" s="52"/>
+      <c r="B158" s="30"/>
+      <c r="C158" s="30"/>
+      <c r="D158" s="30"/>
+      <c r="E158" s="30"/>
+      <c r="F158" s="30"/>
+      <c r="G158" s="30"/>
+      <c r="H158" s="30"/>
+      <c r="I158" s="30"/>
+      <c r="J158" s="30"/>
+      <c r="K158" s="30"/>
+      <c r="L158" s="30"/>
     </row>
     <row r="159" spans="1:12">
       <c r="A159" s="1"/>
-      <c r="B159" s="62"/>
-      <c r="C159" s="62"/>
-      <c r="D159" s="52"/>
-      <c r="E159" s="52"/>
-      <c r="F159" s="52"/>
-      <c r="G159" s="2"/>
-      <c r="H159" s="52"/>
-      <c r="I159" s="52"/>
-      <c r="J159" s="52"/>
-      <c r="K159" s="52"/>
-      <c r="L159" s="52"/>
+      <c r="B159" s="30"/>
+      <c r="C159" s="30"/>
+      <c r="D159" s="30"/>
+      <c r="E159" s="30"/>
+      <c r="F159" s="30"/>
+      <c r="G159" s="30"/>
+      <c r="H159" s="30"/>
+      <c r="I159" s="30"/>
+      <c r="J159" s="30"/>
+      <c r="K159" s="30"/>
+      <c r="L159" s="30"/>
     </row>
     <row r="160" spans="1:12">
       <c r="A160" s="1"/>
-      <c r="B160" s="62"/>
-      <c r="C160" s="62"/>
-      <c r="D160" s="52"/>
-      <c r="E160" s="52"/>
-      <c r="F160" s="52"/>
-      <c r="G160" s="2"/>
-      <c r="H160" s="52"/>
-      <c r="I160" s="52"/>
-      <c r="J160" s="52"/>
-      <c r="K160" s="52"/>
-      <c r="L160" s="52"/>
+      <c r="B160" s="30"/>
+      <c r="C160" s="30"/>
+      <c r="D160" s="30"/>
+      <c r="E160" s="30"/>
+      <c r="F160" s="30"/>
+      <c r="G160" s="30"/>
+      <c r="H160" s="30"/>
+      <c r="I160" s="30"/>
+      <c r="J160" s="30"/>
+      <c r="K160" s="30"/>
+      <c r="L160" s="30"/>
     </row>
     <row r="161" spans="1:12">
       <c r="A161" s="1"/>
-      <c r="B161" s="62"/>
-      <c r="C161" s="62"/>
-      <c r="D161" s="52"/>
-      <c r="E161" s="52"/>
-      <c r="F161" s="52"/>
-      <c r="G161" s="2"/>
-      <c r="H161" s="52"/>
-      <c r="I161" s="52"/>
-      <c r="J161" s="52"/>
-      <c r="K161" s="52"/>
-      <c r="L161" s="52"/>
+      <c r="B161" s="30"/>
+      <c r="C161" s="30"/>
+      <c r="D161" s="30"/>
+      <c r="E161" s="30"/>
+      <c r="F161" s="30"/>
+      <c r="G161" s="30"/>
+      <c r="H161" s="30"/>
+      <c r="I161" s="30"/>
+      <c r="J161" s="30"/>
+      <c r="K161" s="30"/>
+      <c r="L161" s="30"/>
     </row>
     <row r="162" spans="1:12" ht="51" customHeight="1">
       <c r="A162" s="1"/>
-      <c r="B162" s="62"/>
-      <c r="C162" s="62"/>
-      <c r="D162" s="52"/>
-      <c r="E162" s="52"/>
-      <c r="F162" s="52"/>
-      <c r="G162" s="2"/>
-      <c r="H162" s="52"/>
-      <c r="I162" s="52"/>
-      <c r="J162" s="52"/>
-      <c r="K162" s="52"/>
-      <c r="L162" s="52"/>
+      <c r="B162" s="30"/>
+      <c r="C162" s="30"/>
+      <c r="D162" s="30"/>
+      <c r="E162" s="30"/>
+      <c r="F162" s="30"/>
+      <c r="G162" s="30"/>
+      <c r="H162" s="30"/>
+      <c r="I162" s="30"/>
+      <c r="J162" s="30"/>
+      <c r="K162" s="30"/>
+      <c r="L162" s="30"/>
     </row>
     <row r="163" spans="1:12">
       <c r="A163" s="1"/>
-      <c r="B163" s="52" t="s">
+      <c r="B163" s="37" t="s">
         <v>70</v>
       </c>
-      <c r="C163" s="52"/>
-      <c r="D163" s="2"/>
-      <c r="E163" s="2"/>
+      <c r="C163" s="37"/>
+      <c r="D163" s="37"/>
+      <c r="E163" s="37"/>
       <c r="F163" s="2"/>
       <c r="G163" s="2"/>
       <c r="H163" s="2"/>
-      <c r="I163" s="52" t="s">
+      <c r="I163" s="37" t="s">
         <v>71</v>
       </c>
-      <c r="J163" s="52"/>
+      <c r="J163" s="37"/>
       <c r="K163" s="2"/>
       <c r="L163" s="2"/>
     </row>
@@ -4567,15 +4558,15 @@
     </row>
     <row r="168" spans="1:12">
       <c r="A168" s="1"/>
-      <c r="B168" s="52"/>
-      <c r="C168" s="52"/>
+      <c r="B168" s="37"/>
+      <c r="C168" s="37"/>
       <c r="D168" s="2"/>
       <c r="E168" s="2"/>
       <c r="F168" s="2"/>
       <c r="G168" s="2"/>
       <c r="H168" s="2"/>
-      <c r="I168" s="52"/>
-      <c r="J168" s="52"/>
+      <c r="I168" s="37"/>
+      <c r="J168" s="37"/>
       <c r="K168" s="2"/>
       <c r="L168" s="2"/>
     </row>
@@ -4665,77 +4656,100 @@
     </row>
     <row r="175" spans="1:12">
       <c r="A175" s="1"/>
-      <c r="B175" s="53"/>
-      <c r="C175" s="54"/>
-      <c r="D175" s="53"/>
-      <c r="E175" s="59"/>
-      <c r="F175" s="54"/>
-      <c r="G175" s="53"/>
-      <c r="H175" s="59"/>
-      <c r="I175" s="59"/>
-      <c r="J175" s="54"/>
-      <c r="K175" s="53"/>
-      <c r="L175" s="54"/>
+      <c r="B175" s="55"/>
+      <c r="C175" s="56"/>
+      <c r="D175" s="55"/>
+      <c r="E175" s="61"/>
+      <c r="F175" s="56"/>
+      <c r="G175" s="55"/>
+      <c r="H175" s="61"/>
+      <c r="I175" s="61"/>
+      <c r="J175" s="56"/>
+      <c r="K175" s="55"/>
+      <c r="L175" s="56"/>
     </row>
     <row r="176" spans="1:12">
       <c r="A176" s="1"/>
-      <c r="B176" s="55"/>
-      <c r="C176" s="56"/>
-      <c r="D176" s="55"/>
-      <c r="E176" s="60"/>
-      <c r="F176" s="56"/>
-      <c r="G176" s="55"/>
-      <c r="H176" s="60"/>
-      <c r="I176" s="60"/>
-      <c r="J176" s="56"/>
-      <c r="K176" s="55"/>
-      <c r="L176" s="56"/>
+      <c r="B176" s="57"/>
+      <c r="C176" s="58"/>
+      <c r="D176" s="57"/>
+      <c r="E176" s="62"/>
+      <c r="F176" s="58"/>
+      <c r="G176" s="57"/>
+      <c r="H176" s="62"/>
+      <c r="I176" s="62"/>
+      <c r="J176" s="58"/>
+      <c r="K176" s="57"/>
+      <c r="L176" s="58"/>
     </row>
     <row r="177" spans="1:12">
       <c r="A177" s="1"/>
-      <c r="B177" s="57"/>
-      <c r="C177" s="58"/>
-      <c r="D177" s="57"/>
-      <c r="E177" s="61"/>
-      <c r="F177" s="58"/>
-      <c r="G177" s="57"/>
-      <c r="H177" s="61"/>
-      <c r="I177" s="61"/>
-      <c r="J177" s="58"/>
-      <c r="K177" s="57"/>
-      <c r="L177" s="58"/>
+      <c r="B177" s="59"/>
+      <c r="C177" s="60"/>
+      <c r="D177" s="59"/>
+      <c r="E177" s="63"/>
+      <c r="F177" s="60"/>
+      <c r="G177" s="59"/>
+      <c r="H177" s="63"/>
+      <c r="I177" s="63"/>
+      <c r="J177" s="60"/>
+      <c r="K177" s="59"/>
+      <c r="L177" s="60"/>
     </row>
     <row r="178" spans="1:12">
       <c r="A178" s="25"/>
-      <c r="B178" s="35" t="s">
+      <c r="B178" s="38" t="s">
+        <v>31</v>
+      </c>
+      <c r="C178" s="39"/>
+      <c r="D178" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C178" s="36"/>
-      <c r="D178" s="37" t="s">
-        <v>33</v>
-      </c>
-      <c r="E178" s="38"/>
-      <c r="F178" s="39"/>
-      <c r="G178" s="40" t="s">
+      <c r="E178" s="41"/>
+      <c r="F178" s="42"/>
+      <c r="G178" s="43" t="s">
         <v>72</v>
       </c>
-      <c r="H178" s="41"/>
-      <c r="I178" s="41"/>
-      <c r="J178" s="42"/>
-      <c r="K178" s="43" t="s">
-        <v>35</v>
-      </c>
-      <c r="L178" s="44"/>
+      <c r="H178" s="44"/>
+      <c r="I178" s="44"/>
+      <c r="J178" s="45"/>
+      <c r="K178" s="46" t="s">
+        <v>34</v>
+      </c>
+      <c r="L178" s="47"/>
     </row>
     <row r="187" spans="1:12" ht="30" customHeight="1"/>
     <row r="188" spans="1:12" ht="30" customHeight="1"/>
-    <row r="190" spans="1:12" ht="27" customHeight="1"/>
-    <row r="191" spans="1:12" ht="27" customHeight="1"/>
+    <row r="190" spans="1:12" ht="30" customHeight="1"/>
+    <row r="191" spans="1:12" ht="30" customHeight="1"/>
+    <row r="192" spans="1:12" ht="30" customHeight="1"/>
   </sheetData>
-  <mergeCells count="176">
-    <mergeCell ref="D6:F6"/>
+  <mergeCells count="167">
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="J20:J21"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D19"/>
+    <mergeCell ref="G28:I28"/>
+    <mergeCell ref="J28:L28"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="J26:L26"/>
+    <mergeCell ref="D20:D22"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="B152:E152"/>
+    <mergeCell ref="G152:L152"/>
+    <mergeCell ref="D32:L32"/>
+    <mergeCell ref="B33:L33"/>
     <mergeCell ref="B116:J119"/>
     <mergeCell ref="K116:L119"/>
+    <mergeCell ref="L20:L21"/>
+    <mergeCell ref="B24:L24"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="B36:L46"/>
+    <mergeCell ref="E48:L48"/>
+    <mergeCell ref="C74:L74"/>
+    <mergeCell ref="K60:L60"/>
     <mergeCell ref="D5:F5"/>
     <mergeCell ref="C8:L8"/>
     <mergeCell ref="C9:L10"/>
@@ -4755,35 +4769,19 @@
     <mergeCell ref="K55:L55"/>
     <mergeCell ref="C30:L30"/>
     <mergeCell ref="B31:L31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="J27:L27"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="L17:L18"/>
     <mergeCell ref="B53:L53"/>
     <mergeCell ref="B54:C54"/>
     <mergeCell ref="D54:F54"/>
     <mergeCell ref="G54:J54"/>
     <mergeCell ref="K54:L54"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="J27:L27"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="D20:D22"/>
-    <mergeCell ref="L20:L21"/>
-    <mergeCell ref="B24:L24"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="J20:J21"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D19"/>
-    <mergeCell ref="G28:I28"/>
-    <mergeCell ref="J28:L28"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="J26:L26"/>
-    <mergeCell ref="D32:L32"/>
-    <mergeCell ref="B33:L33"/>
-    <mergeCell ref="B36:L46"/>
-    <mergeCell ref="E48:L48"/>
-    <mergeCell ref="C74:L74"/>
+    <mergeCell ref="B87:J87"/>
+    <mergeCell ref="K87:L87"/>
+    <mergeCell ref="B88:J88"/>
+    <mergeCell ref="K88:L88"/>
     <mergeCell ref="C75:G75"/>
     <mergeCell ref="J76:L76"/>
     <mergeCell ref="B80:L80"/>
@@ -4799,11 +4797,6 @@
     <mergeCell ref="B60:C60"/>
     <mergeCell ref="D60:F60"/>
     <mergeCell ref="G60:J60"/>
-    <mergeCell ref="K60:L60"/>
-    <mergeCell ref="B87:J87"/>
-    <mergeCell ref="K87:L87"/>
-    <mergeCell ref="B88:J88"/>
-    <mergeCell ref="K88:L88"/>
     <mergeCell ref="B89:J89"/>
     <mergeCell ref="K89:L89"/>
     <mergeCell ref="C83:E83"/>
@@ -4860,6 +4853,7 @@
     <mergeCell ref="K109:L109"/>
     <mergeCell ref="B110:J110"/>
     <mergeCell ref="K110:L110"/>
+    <mergeCell ref="J137:L137"/>
     <mergeCell ref="B124:C124"/>
     <mergeCell ref="D124:F124"/>
     <mergeCell ref="G124:J124"/>
@@ -4874,17 +4868,7 @@
     <mergeCell ref="D121:F123"/>
     <mergeCell ref="G121:J123"/>
     <mergeCell ref="K121:L123"/>
-    <mergeCell ref="B143:B150"/>
-    <mergeCell ref="C143:D150"/>
-    <mergeCell ref="E143:F150"/>
-    <mergeCell ref="G143:I150"/>
-    <mergeCell ref="J143:L150"/>
-    <mergeCell ref="C135:G135"/>
-    <mergeCell ref="C136:D136"/>
-    <mergeCell ref="F136:G136"/>
-    <mergeCell ref="J136:L136"/>
-    <mergeCell ref="C137:G137"/>
-    <mergeCell ref="J137:L137"/>
+    <mergeCell ref="B163:E163"/>
     <mergeCell ref="B178:C178"/>
     <mergeCell ref="D178:F178"/>
     <mergeCell ref="G178:J178"/>
@@ -4901,19 +4885,20 @@
     <mergeCell ref="D175:F177"/>
     <mergeCell ref="G175:J177"/>
     <mergeCell ref="K175:L177"/>
-    <mergeCell ref="B152:C152"/>
-    <mergeCell ref="I152:J152"/>
-    <mergeCell ref="B156:C162"/>
-    <mergeCell ref="D156:F162"/>
-    <mergeCell ref="H156:L162"/>
-    <mergeCell ref="B163:C163"/>
     <mergeCell ref="I163:J163"/>
     <mergeCell ref="B140:L140"/>
+    <mergeCell ref="C135:G135"/>
+    <mergeCell ref="C136:D136"/>
+    <mergeCell ref="F136:G136"/>
+    <mergeCell ref="J136:L136"/>
+    <mergeCell ref="C137:G137"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="portrait"/>
-  <rowBreaks count="2" manualBreakCount="2">
+  <rowBreaks count="4" manualBreakCount="4">
+    <brk id="62" max="16383" man="1"/>
     <brk id="63" max="16383" man="1"/>
+    <brk id="126" max="16383" man="1"/>
     <brk id="127" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>

</xml_diff>